<commit_message>
fix(rag): guard use_summary on multi-facet single-course queries
When the LLM emits use_summary=True for a mixed-intent query like Q2
("is this class good for me + main topics, methods, models"), the router
discards the 4 fanned-out subqueries and pins the result to course_summary
(one pinned doc, no rerank). Multi-facet fanout on a single course is
incompatible with a single summary doc.

Add a deterministic repair in _validate_and_repair: if use_summary=True
AND len(subqueries) >= 2 AND len(course_ids) == 1, flip use_summary=False
and log repair "use_summary_reset_multifacet".

Q2 affected-only eval (curated20_v2_q2_use_summary_guard_20260521):
- function: course_summary -> hybrid_course
- context_recall: 0.0 -> 1.0
- context_precision: 0.833 -> 0.5 (expected; 5 chunks vs 3)
- Router accuracy lifts curated20_v2 from 19/20 to 20/20.
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/ragas_20260519_curated20_v2.xlsx
+++ b/tamu_data/evals/golden_sets/ragas_20260519_curated20_v2.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,21 @@
           <t>run:curated20_v2_cap4_20260521_20260521_200401:context_recall</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>run:curated20_v2_q2_use_summary_guard_20260521</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>run:curated20_v2_q2_use_summary_guard_20260521:context_precision</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>run:curated20_v2_q2_use_summary_guard_20260521:context_recall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -636,6 +651,17 @@
       </c>
       <c r="R3" t="n">
         <v>0</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ISEN 620 0.65, ISEN 620 0.58, ISEN 620 0.57, ISEN 620 0.64, ISEN 620 0.65</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">

</xml_diff>